<commit_message>
fix(dashboard): correct Nifty 50 universe (swap 6 stale constituents)
Replace 6 stocks no longer in the official Nifty 50 index (DIVISLAB,
BPCL, BRITANNIA, HEROMOTOCO, INDUSINDBK, TATAMOTORS) with the current
6 (ETERNAL, INDIGO, JIOFIN, MAXHEALTH, TMPV, TRENT) across all quarters,
RBI policy behaviour, the 211 F&O universe's is_nifty50 flags, and the
Dussehra/Diwali/Christmas holiday events. Direction/window/win-rate for
the 6 new stocks were freshly backtested from real NSE price history
using the same walk-forward methodology as the other 44, not copied or
guessed.

The already-executed Mahatma Gandhi Jayanti (2 Oct) event is left
completely untouched, since that trade window is already live.

Also simplifies "17-Quarter" labels in the dashboard UI to just
"Quarter" per user feedback, and points rebuild_perfect_dashboard_data.py
at the current NSE snapshot CSV with lot sizes for the 6 new stocks.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Nifty50Stocks_QtyResultDates.xlsx
+++ b/Nifty50Stocks_QtyResultDates.xlsx
@@ -21,9 +21,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -3964,16 +3963,16 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Hero MotoCorp Ltd.</t>
+          <t>InterGlobe Aviation Ltd.</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
-          <t>HEROMOTOCO</t>
+          <t>INDIGO</t>
         </is>
       </c>
       <c r="C21" s="10" t="n">
-        <v>45875</v>
+        <v>45868</v>
       </c>
     </row>
     <row r="22">
@@ -4024,16 +4023,16 @@
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>IndusInd Bank Ltd.</t>
+          <t>Max Healthcare Institute Ltd.</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
-          <t>INDUSINDBK</t>
+          <t>MAXHEALTH</t>
         </is>
       </c>
       <c r="C25" s="10" t="n">
-        <v>45866</v>
+        <v>45882</v>
       </c>
     </row>
     <row r="26">
@@ -4309,12 +4308,12 @@
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>Tata Motors Ltd.</t>
+          <t>Tata Motors Passenger Vehicles Ltd.</t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
-          <t>TATAMOTORS</t>
+          <t>TMPV</t>
         </is>
       </c>
       <c r="C44" s="10" t="n">

</xml_diff>